<commit_message>
feat: add battle pass rewards and GM support
</commit_message>
<xml_diff>
--- a/config/xlsx/activities.xlsx
+++ b/config/xlsx/activities.xlsx
@@ -1,37 +1,190 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="17680" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="activities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="22">
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -40,12 +193,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -54,14 +393,265 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,8 +665,56 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -429,7 +1067,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -439,15 +1076,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="4"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="1" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,6 +1111,11 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>widget</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>enabled</t>
         </is>
       </c>
     </row>
@@ -542,6 +1179,39 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>首期战令</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01T00:00:00+08:00</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01T00:00:00+08:00</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>BattlePass</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add activities and inventory updates with recipe and crafting fixes
</commit_message>
<xml_diff>
--- a/config/xlsx/activities.xlsx
+++ b/config/xlsx/activities.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activities" sheetId="1" r:id="R8b78cdc6641f4508"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activities" sheetId="1" r:id="R65dace859e2d44b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,9 +13,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="@"/>
-  </x:numFmts>
   <x:fonts count="22">
     <x:font>
       <x:sz val="11"/>
@@ -403,20 +400,20 @@
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="49">
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <x:xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
+    <x:xf numFmtId="43" fontId="21" fillId="0" borderId="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="44" fontId="21" fillId="0" borderId="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="41" fontId="21" fillId="0" borderId="0" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="42" fontId="21" fillId="0" borderId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
@@ -425,7 +422,7 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="21" fillId="3" borderId="2" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
@@ -549,7 +546,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -560,10 +557,21 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
     <x:cellStyle name="常规" xfId="0"/>
@@ -685,6 +693,23 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -900,143 +925,225 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
-  <cols>
-    <col min="1" max="6" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cycle</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">start_time</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">end_time</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">widget</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">enabled</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>每日合成</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="3" t="str"/>
-      <c r="G2"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>限时活动</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-10T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-20T00:00:00Z</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="str"/>
-      <c r="G3"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>周常任务</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="3" t="str">
-        <v>WeeklyActivityEntry</v>
-      </c>
-      <c r="G4"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>首期战令</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="3" t="str">
-        <v>BattlePass</v>
-      </c>
-      <c r="G5" s="3" t="str">
-        <v>TRUE</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>万象仙册</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" t="str">
-        <v>CardCollection</v>
-      </c>
-      <c r="G6" t="str">
-        <v>TRUE</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <x:cols>
+    <x:col min="1" max="6" width="16" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">id</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">name</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">cycle</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">start_time</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">end_time</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">widget</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G1" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">enabled</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">config</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每日合成</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="n"/>
+      <x:c r="E2" s="6" t="n"/>
+      <x:c r="F2" s="3" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">限时活动</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="3" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-07-10T00:00:00Z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="6" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-07-20T00:00:00Z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="3" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">周常任务</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="n"/>
+      <x:c r="E4" s="6" t="n"/>
+      <x:c r="F4" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">WeeklyActivityEntry</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="2" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">首期战令</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="3" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="n"/>
+      <x:c r="E5" s="6" t="n"/>
+      <x:c r="F5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">BattlePass</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">TRUE</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">万象仙册</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="n"/>
+      <x:c r="E6" s="7" t="n"/>
+      <x:c r="F6" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CardCollection</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">TRUE</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">爬天梯</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-07T16:00:00Z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-10T16:00:00Z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">StairClimb</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">TRUE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">{"group_size":20,"bot_min_minutes":30,"bot_max_minutes":90,"rewards":[{"min_rank":1,"max_rank":1,"stamina":300,"spirit_stones":3000},{"min_rank":2,"max_rank":2,"stamina":275,"spirit_stones":2750},{"min_rank":3,"max_rank":3,"stamina":250,"spirit_stones":2500},{"min_rank":4,"max_rank":4,"stamina":225,"spirit_stones":2250},{"min_rank":5,"max_rank":5,"stamina":200,"spirit_stones":2000},{"min_rank":6,"max_rank":6,"stamina":175,"spirit_stones":1750},{"min_rank":7,"max_rank":7,"stamina":150,"spirit_stones":1500},{"min_rank":8,"max_rank":8,"stamina":125,"spirit_stones":1250},{"min_rank":9,"max_rank":9,"stamina":100,"spirit_stones":1000},{"min_rank":10,"max_rank":10,"stamina":75,"spirit_stones":750},{"min_rank":11,"max_rank":20,"stamina":50,"spirit_stones":500}],"order_points_ratio":0.1,"bot_order_value":100}</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>订单补给</x:v>
+      </x:c>
+      <x:c r="C8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+      <x:c r="F8" t="str">
+        <x:v>OrderSupply</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>{"target_count":5,"reward_count":3}</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update gameplay, activities, configuration and GM controls
</commit_message>
<xml_diff>
--- a/config/xlsx/activities.xlsx
+++ b/config/xlsx/activities.xlsx
@@ -2,18 +2,100 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activities" sheetId="1" r:id="R65dace859e2d44b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activities" sheetId="1" r:id="R9d3ea59853794b6d"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:si>
+    <x:t xml:space="preserve">id</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">name</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">cycle</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">start_time</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">end_time</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">widget</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">enabled</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">config</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">限时活动</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-10T00:00:00Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-07-20T00:00:00Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">11</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">周常任务</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">WeeklyActivityEntry</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">首期战令</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">BattlePass</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">TRUE</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">万象仙册</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">CardCollection</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">爬天梯</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-10-07T16:00:00Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">2026-10-10T16:00:00Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">StairClimb</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">订单补给</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">OrderSupply</x:t>
+  </x:si>
+</x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="22">
+  <x:numFmts count="4">
+    <x:numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <x:numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </x:numFmts>
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -23,11 +105,6 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="宋体"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
       <x:name val="宋体"/>
     </x:font>
     <x:font>
@@ -93,19 +170,13 @@
       <x:name val="宋体"/>
     </x:font>
     <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFA7D00"/>
+      <x:name val="宋体"/>
+    </x:font>
+    <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="宋体"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FFFA7D00"/>
-      <x:name val="宋体"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
       <x:color theme="1"/>
       <x:name val="宋体"/>
     </x:font>
@@ -127,11 +198,6 @@
     <x:font>
       <x:sz val="11"/>
       <x:color theme="0"/>
-      <x:name val="宋体"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color theme="1"/>
       <x:name val="宋体"/>
     </x:font>
   </x:fonts>
@@ -304,7 +370,13 @@
     </x:fill>
   </x:fills>
   <x:borders count="10">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
     <x:border>
       <x:left style="thin">
         <x:color auto="1"/>
@@ -318,6 +390,7 @@
       <x:bottom style="thin">
         <x:color auto="1"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -332,16 +405,25 @@
       <x:bottom style="thin">
         <x:color rgb="FFB2B2B2"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
       <x:bottom style="medium">
         <x:color theme="4"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
       <x:bottom style="medium">
         <x:color theme="4" tint="0.49998"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -356,6 +438,7 @@
       <x:bottom style="thin">
         <x:color rgb="FF7F7F7F"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -370,6 +453,7 @@
       <x:bottom style="thin">
         <x:color rgb="FF3F3F3F"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="double">
@@ -384,194 +468,191 @@
       <x:bottom style="double">
         <x:color rgb="FF3F3F3F"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
       <x:bottom style="double">
         <x:color rgb="FFFF8001"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
       <x:top style="thin">
         <x:color theme="4"/>
       </x:top>
       <x:bottom style="double">
         <x:color theme="4"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="49">
-    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0"/>
-    <x:xf numFmtId="43" fontId="21" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="44" fontId="21" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="9" fontId="21" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="41" fontId="21" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="42" fontId="21" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="3" borderId="2" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <x:xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="2">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="4">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="5">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="6">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="5" borderId="5">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="7">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="8">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="9">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="7" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="9" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="10" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="14" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="17" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="21" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="22" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="29" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="30" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="33" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
+    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
+    <x:xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </x:cellXfs>
   <x:cellStyles count="49">
     <x:cellStyle name="常规" xfId="0"/>
@@ -624,92 +705,187 @@
     <x:cellStyle name="40% - 强调文字颜色 6" xfId="47"/>
     <x:cellStyle name="60% - 强调文字颜色 6" xfId="48"/>
   </x:cellStyles>
-  <x:colors>
-    <x:indexedColors>
-      <x:rgbColor rgb="00000000"/>
-      <x:rgbColor rgb="00FFFFFF"/>
-      <x:rgbColor rgb="00FF0000"/>
-      <x:rgbColor rgb="0000FF00"/>
-      <x:rgbColor rgb="000000FF"/>
-      <x:rgbColor rgb="00FFFF00"/>
-      <x:rgbColor rgb="00FF00FF"/>
-      <x:rgbColor rgb="0000FFFF"/>
-      <x:rgbColor rgb="00000000"/>
-      <x:rgbColor rgb="00FFFFFF"/>
-      <x:rgbColor rgb="00FF0000"/>
-      <x:rgbColor rgb="0000FF00"/>
-      <x:rgbColor rgb="000000FF"/>
-      <x:rgbColor rgb="00FFFF00"/>
-      <x:rgbColor rgb="00FF00FF"/>
-      <x:rgbColor rgb="0000FFFF"/>
-      <x:rgbColor rgb="00800000"/>
-      <x:rgbColor rgb="00008000"/>
-      <x:rgbColor rgb="00000080"/>
-      <x:rgbColor rgb="00808000"/>
-      <x:rgbColor rgb="00800080"/>
-      <x:rgbColor rgb="00008080"/>
-      <x:rgbColor rgb="00C0C0C0"/>
-      <x:rgbColor rgb="00808080"/>
-      <x:rgbColor rgb="009999FF"/>
-      <x:rgbColor rgb="00993366"/>
-      <x:rgbColor rgb="00FFFFCC"/>
-      <x:rgbColor rgb="00CCFFFF"/>
-      <x:rgbColor rgb="00660066"/>
-      <x:rgbColor rgb="00FF8080"/>
-      <x:rgbColor rgb="000066CC"/>
-      <x:rgbColor rgb="00CCCCFF"/>
-      <x:rgbColor rgb="00000080"/>
-      <x:rgbColor rgb="00FF00FF"/>
-      <x:rgbColor rgb="00FFFF00"/>
-      <x:rgbColor rgb="0000FFFF"/>
-      <x:rgbColor rgb="00800080"/>
-      <x:rgbColor rgb="00800000"/>
-      <x:rgbColor rgb="00008080"/>
-      <x:rgbColor rgb="000000FF"/>
-      <x:rgbColor rgb="0000CCFF"/>
-      <x:rgbColor rgb="00CCFFFF"/>
-      <x:rgbColor rgb="00CCFFCC"/>
-      <x:rgbColor rgb="00FFFF99"/>
-      <x:rgbColor rgb="0099CCFF"/>
-      <x:rgbColor rgb="00FF99CC"/>
-      <x:rgbColor rgb="00CC99FF"/>
-      <x:rgbColor rgb="00FFCC99"/>
-      <x:rgbColor rgb="003366FF"/>
-      <x:rgbColor rgb="0033CCCC"/>
-      <x:rgbColor rgb="0099CC00"/>
-      <x:rgbColor rgb="00FFCC00"/>
-      <x:rgbColor rgb="00FF9900"/>
-      <x:rgbColor rgb="00FF6600"/>
-      <x:rgbColor rgb="00666699"/>
-      <x:rgbColor rgb="00969696"/>
-      <x:rgbColor rgb="00003366"/>
-      <x:rgbColor rgb="00339966"/>
-      <x:rgbColor rgb="00003300"/>
-      <x:rgbColor rgb="00333300"/>
-      <x:rgbColor rgb="00993300"/>
-      <x:rgbColor rgb="00993366"/>
-      <x:rgbColor rgb="00333399"/>
-      <x:rgbColor rgb="00333333"/>
-    </x:indexedColors>
-  </x:colors>
+  <x:dxfs count="17">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="1"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="1"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="1"/>
+      </x:font>
+      <x:border>
+        <x:top style="double">
+          <x:color theme="4"/>
+        </x:top>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="0"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color theme="1"/>
+      </x:font>
+      <x:border>
+        <x:left style="thin">
+          <x:color theme="4"/>
+        </x:left>
+        <x:right style="thin">
+          <x:color theme="4"/>
+        </x:right>
+        <x:top style="thin">
+          <x:color theme="4"/>
+        </x:top>
+        <x:bottom style="thin">
+          <x:color theme="4"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+      <x:border>
+        <x:bottom style="thin">
+          <x:color theme="4" tint="0.39998"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+      <x:border>
+        <x:bottom style="thin">
+          <x:color theme="4" tint="0.39998"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color theme="1"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color theme="1"/>
+      </x:font>
+      <x:border>
+        <x:bottom style="thin">
+          <x:color theme="4" tint="0.39998"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="1"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="1"/>
+      </x:font>
+      <x:border>
+        <x:top style="thin">
+          <x:color theme="4"/>
+        </x:top>
+        <x:bottom style="thin">
+          <x:color theme="4"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="1"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+      <x:border>
+        <x:top style="thin">
+          <x:color theme="4" tint="0.39998"/>
+        </x:top>
+        <x:bottom style="thin">
+          <x:color theme="4" tint="0.39998"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color theme="1"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor theme="4" tint="0.79998"/>
+        </x:patternFill>
+      </x:fill>
+      <x:border>
+        <x:bottom style="thin">
+          <x:color theme="4" tint="0.39998"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
-</file>
-
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <xfpb:bag type="Checkbox"/>
-  <xfpb:bag type="XFControls">
-    <xfpb:bagId k="CellControl">0</xfpb:bagId>
-  </xfpb:bag>
-  <xfpb:bag type="XFComplement">
-    <xfpb:bagId k="XFControls">1</xfpb:bagId>
-  </xfpb:bag>
-  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <xfpb:a k="MappedFeaturePropertyBags">
-      <xfpb:bagId>2</xfpb:bagId>
-    </xfpb:a>
-  </xfpb:bag>
-</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -926,207 +1102,159 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <x:sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <x:cols>
     <x:col min="1" max="6" width="16" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">id</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">name</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cycle</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">start_time</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">end_time</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">widget</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">enabled</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">config</x:t>
-        </x:is>
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H1" t="s">
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">每日合成</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="3" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D2" s="6" t="n"/>
-      <x:c r="E2" s="6" t="n"/>
-      <x:c r="F2" s="3" t="str"/>
+      <x:c r="A2" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C2" s="3">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E2" s="4" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F2" s="3" t="s">
+        <x:v>11</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="2" t="n">
+      <x:c r="A3" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C3" s="3">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">限时活动</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="3" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D3" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-10T00:00:00Z</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-20T00:00:00Z</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F3" s="3" t="str"/>
+      <x:c r="D3" s="4"/>
+      <x:c r="E3" s="4"/>
+      <x:c r="F3" s="3" t="s">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="2" t="n">
+      <x:c r="A4" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C4" s="3">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周常任务</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="3" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D4" s="6" t="n"/>
-      <x:c r="E4" s="6" t="n"/>
-      <x:c r="F4" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">WeeklyActivityEntry</x:t>
-        </x:is>
+      <x:c r="D4" s="4"/>
+      <x:c r="E4" s="4"/>
+      <x:c r="F4" s="3" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G4" s="3" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="2" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">首期战令</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="3" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="n"/>
-      <x:c r="E5" s="6" t="n"/>
-      <x:c r="F5" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BattlePass</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G5" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TRUE</x:t>
-        </x:is>
+      <x:c r="A5">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C5">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D5" s="5"/>
+      <x:c r="E5" s="5"/>
+      <x:c r="F5" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G5" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">万象仙册</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" t="n">
+      <x:c r="A6">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B6" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C6">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="n"/>
-      <x:c r="E6" s="7" t="n"/>
-      <x:c r="F6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CardCollection</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TRUE</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="D6" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E6" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F6" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G6" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H6"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">爬天梯</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" t="n">
+      <x:c r="A7">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B7" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C7">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-07T16:00:00Z</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-10T16:00:00Z</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">StairClimb</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TRUE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">{"group_size":20,"bot_min_minutes":30,"bot_max_minutes":90,"rewards":[{"min_rank":1,"max_rank":1,"stamina":300,"spirit_stones":3000},{"min_rank":2,"max_rank":2,"stamina":275,"spirit_stones":2750},{"min_rank":3,"max_rank":3,"stamina":250,"spirit_stones":2500},{"min_rank":4,"max_rank":4,"stamina":225,"spirit_stones":2250},{"min_rank":5,"max_rank":5,"stamina":200,"spirit_stones":2000},{"min_rank":6,"max_rank":6,"stamina":175,"spirit_stones":1750},{"min_rank":7,"max_rank":7,"stamina":150,"spirit_stones":1500},{"min_rank":8,"max_rank":8,"stamina":125,"spirit_stones":1250},{"min_rank":9,"max_rank":9,"stamina":100,"spirit_stones":1000},{"min_rank":10,"max_rank":10,"stamina":75,"spirit_stones":750},{"min_rank":11,"max_rank":20,"stamina":50,"spirit_stones":500}],"order_points_ratio":0.1,"bot_order_value":100}</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="F7" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>订单补给</x:v>
+        <x:v>订单对战</x:v>
       </x:c>
       <x:c r="C8" t="n">
         <x:v>0</x:v>
@@ -1134,14 +1262,32 @@
       <x:c r="D8"/>
       <x:c r="E8"/>
       <x:c r="F8" t="str">
-        <x:v>OrderSupply</x:v>
+        <x:v>OrderDuel</x:v>
       </x:c>
       <x:c r="G8" t="str">
         <x:v>TRUE</x:v>
       </x:c>
-      <x:c r="H8" t="str">
-        <x:v>{"target_count":5,"reward_count":3}</x:v>
-      </x:c>
+      <x:c r="H8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>剑墟秘境</x:v>
+      </x:c>
+      <x:c r="C9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
+      <x:c r="F9" t="str">
+        <x:v>SecretRealm</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+      <x:c r="H9"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>